<commit_message>
Update Xenium SpD annotaitons (xL1_Inhib, xLD_glia, xVasc.mural) in table
</commit_message>
<xml_diff>
--- a/processed-data/21_Xenium/13.1_xenium_compare_bansky_clusters/banksy_clustering_annotation_k11_summary.xlsx
+++ b/processed-data/21_Xenium/13.1_xenium_compare_bansky_clusters/banksy_clustering_annotation_k11_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lieberinstitute-my.sharepoint.com/personal/louise_huuki_libd_org/Documents/LIBD_code/LFF_spatial_ERC/processed-data/21_Xenium/13.1_xenium_compare_bansky_clusters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="78" documentId="8_{A3DE8289-B4D8-0B48-BA93-A1E439C2703E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1CD7A4D9-B516-0E4B-89EC-B70AC700ED38}"/>
+  <xr:revisionPtr revIDLastSave="89" documentId="8_{A3DE8289-B4D8-0B48-BA93-A1E439C2703E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1DACB192-08BE-DE40-BBA4-EC33BDDB0AF6}"/>
   <bookViews>
-    <workbookView xWindow="36060" yWindow="2280" windowWidth="22340" windowHeight="17180" xr2:uid="{76241F0D-2465-BD4B-8A74-F93DEE6FB35C}"/>
+    <workbookView xWindow="36060" yWindow="2280" windowWidth="32480" windowHeight="17180" xr2:uid="{76241F0D-2465-BD4B-8A74-F93DEE6FB35C}"/>
   </bookViews>
   <sheets>
     <sheet name="banksy_clustering_annotation_k1" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="97">
   <si>
     <t>cluster</t>
   </si>
@@ -187,12 +187,6 @@
     <t>L2</t>
   </si>
   <si>
-    <t>Inhib</t>
-  </si>
-  <si>
-    <t>LD</t>
-  </si>
-  <si>
     <t>WMd</t>
   </si>
   <si>
@@ -298,20 +292,29 @@
     <t xml:space="preserve">interspersed in GM layers </t>
   </si>
   <si>
-    <t>Vasc.adj</t>
-  </si>
-  <si>
-    <t>Vasc.im</t>
-  </si>
-  <si>
-    <t>Vasc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mural/pericyte layer - claude
+    <t>Perivascular immune niche'</t>
+  </si>
+  <si>
+    <t>Vasc_im</t>
+  </si>
+  <si>
+    <t>Vasc_mural</t>
+  </si>
+  <si>
+    <t>Vasc_adj</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mural/pericyte layer
 looks like main blood vessles to us </t>
   </si>
   <si>
-    <t>Perivascular immune niche'</t>
+    <t>LD_glia</t>
+  </si>
+  <si>
+    <t>L1_inhib</t>
+  </si>
+  <si>
+    <t>Layer 1 position + Inhib.Pax6, VIP, and Lamp5 enrichment</t>
   </si>
 </sst>
 </file>
@@ -1207,7 +1210,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E1" t="s">
         <v>3</v>
@@ -1216,13 +1219,13 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
+        <v>58</v>
+      </c>
+      <c r="H1" t="s">
+        <v>59</v>
+      </c>
+      <c r="I1" t="s">
         <v>60</v>
-      </c>
-      <c r="H1" t="s">
-        <v>61</v>
-      </c>
-      <c r="I1" t="s">
-        <v>62</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>50</v>
@@ -1231,7 +1234,7 @@
         <v>51</v>
       </c>
       <c r="L1" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
@@ -1254,22 +1257,22 @@
         <v>9</v>
       </c>
       <c r="G2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="H2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="J2" s="1">
         <v>1</v>
       </c>
       <c r="K2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="51" x14ac:dyDescent="0.2">
@@ -1292,22 +1295,22 @@
         <v>12</v>
       </c>
       <c r="G3" t="s">
+        <v>77</v>
+      </c>
+      <c r="H3" t="s">
+        <v>78</v>
+      </c>
+      <c r="I3" t="s">
         <v>79</v>
-      </c>
-      <c r="H3" t="s">
-        <v>80</v>
-      </c>
-      <c r="I3" t="s">
-        <v>81</v>
       </c>
       <c r="J3" s="1">
         <v>0</v>
       </c>
       <c r="K3" t="s">
+        <v>91</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <v>93</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
@@ -1330,22 +1333,22 @@
         <v>41</v>
       </c>
       <c r="G4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="H4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="I4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="J4" s="1">
         <v>6</v>
       </c>
       <c r="K4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="L4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
@@ -1368,13 +1371,13 @@
         <v>16</v>
       </c>
       <c r="G5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="H5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="I5" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="J5" s="1">
         <v>2</v>
@@ -1385,72 +1388,75 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="B6" t="s">
         <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="D6" s="1">
         <v>2</v>
       </c>
       <c r="E6" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="F6" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="G6" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="H6" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="I6" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="J6" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K6" t="s">
-        <v>53</v>
+        <v>95</v>
+      </c>
+      <c r="L6" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="B7" t="s">
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="D7" s="1">
         <v>3</v>
       </c>
       <c r="E7" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="F7" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="G7" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="H7" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="I7" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="J7" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
@@ -1473,19 +1479,19 @@
         <v>49</v>
       </c>
       <c r="G8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="H8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="I8" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="J8" s="1">
         <v>5</v>
       </c>
       <c r="K8" t="s">
-        <v>55</v>
+        <v>94</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
@@ -1508,19 +1514,19 @@
         <v>32</v>
       </c>
       <c r="G9" t="s">
+        <v>61</v>
+      </c>
+      <c r="H9" t="s">
+        <v>62</v>
+      </c>
+      <c r="I9" t="s">
         <v>63</v>
-      </c>
-      <c r="H9" t="s">
-        <v>64</v>
-      </c>
-      <c r="I9" t="s">
-        <v>65</v>
       </c>
       <c r="J9" s="1">
         <v>7</v>
       </c>
       <c r="K9" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
@@ -1543,19 +1549,19 @@
         <v>28</v>
       </c>
       <c r="G10" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="H10" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="I10" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="J10" s="1">
         <v>8</v>
       </c>
       <c r="K10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
@@ -1578,19 +1584,19 @@
         <v>24</v>
       </c>
       <c r="G11" t="s">
+        <v>66</v>
+      </c>
+      <c r="H11" t="s">
+        <v>67</v>
+      </c>
+      <c r="I11" t="s">
         <v>68</v>
-      </c>
-      <c r="H11" t="s">
-        <v>69</v>
-      </c>
-      <c r="I11" t="s">
-        <v>70</v>
       </c>
       <c r="J11" s="1">
         <v>9</v>
       </c>
       <c r="K11" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
@@ -1613,19 +1619,19 @@
         <v>20</v>
       </c>
       <c r="G12" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="H12" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="I12" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="J12" s="1">
         <v>10</v>
       </c>
       <c r="K12" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>